<commit_message>
feat: reshape demo dataset to Excel codes with template tenant contracts
- Buildings T17 / S9 / G1 (one per house type T/S/G), rooms {no}{building}
  (201T17, 302S9, 102G1); all dependent IDs follow; schema 13 reseeds old saves
- Per-building fee schemes from the Excel invoice sheets (T17 = contract template
  fees; CLEAN/WASH fee types; P&L maps vệ sinh/thang máy/máy giặt/xe điện lines)
- Teams per org chart (VP/VH1/VH2/KD with kind), sales/market staff, allowance split
- Commission ledger per new contract (agency/CTV/sale), repair log with payer,
  supplier contract codes; fix PS-/DC- ID collisions (TPP-/TK-/DCL-)
- Tenant contracts fully filled per Hop_dong_thue_phong_demo_day_du.pdf and
  cross-checked with invoices, deposits, readings and receipts; read-only
  "Xem bản hợp đồng theo mẫu" view; OCR sample driven by data
- Regenerate frozen reports, schema-13 baseline, QA suites and dataset docs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/dataset/report-seed.xlsx
+++ b/docs/qa/dataset/report-seed.xlsx
@@ -87,14 +87,14 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">BÁO CÁO KINH DOANH CẦU GIẤY THÁNG 9/2026</t>
+          <t xml:space="preserve">BÁO CÁO KINH DOANH T17 THÁNG 9/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Bản BC04-202609-CG-v1 · v1 · tạo 2026-10-06 09:00 bởi Hoàng Thu Hà · MAU-G1 · v1 (G1.31.8.26.xlsx) · RPT-ENGINE v1 · pnl.js schema 12 · chế độ Tổng theo mẫu · ô tỷ lệ trống = không áp dụng (mẫu số 0)</t>
+          <t xml:space="preserve">Bản BC04-202609-T17-v1 · v1 · tạo 2026-10-06 09:00 bởi Hoàng Thu Hà · MAU-G1 · v1 (G1.31.8.26.xlsx) · RPT-ENGINE v1 · pnl.js schema 12 · chế độ Tổng theo mẫu · ô tỷ lệ trống = không áp dụng (mẫu số 0)</t>
         </is>
       </c>
     </row>
@@ -132,7 +132,7 @@
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="4">
-        <v>33006600</v>
+        <v>32338000</v>
       </c>
       <c r="D6" s="1"/>
     </row>
@@ -160,7 +160,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-401</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
     </row>
@@ -176,7 +176,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-401</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
     </row>
@@ -216,7 +216,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-401</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
     </row>
@@ -248,7 +248,7 @@
         </is>
       </c>
       <c r="C15" s="2">
-        <v>3256600</v>
+        <v>3428000</v>
       </c>
       <c r="D15"/>
     </row>
@@ -260,7 +260,7 @@
         </is>
       </c>
       <c r="C16" s="2">
-        <v>1170000</v>
+        <v>1080000</v>
       </c>
       <c r="D16"/>
     </row>
@@ -272,7 +272,7 @@
         </is>
       </c>
       <c r="C17" s="2">
-        <v>300000</v>
+        <v>360000</v>
       </c>
       <c r="D17"/>
     </row>
@@ -296,7 +296,7 @@
         </is>
       </c>
       <c r="C19" s="2">
-        <v>1080000</v>
+        <v>150000</v>
       </c>
       <c r="D19"/>
     </row>
@@ -308,7 +308,7 @@
         </is>
       </c>
       <c r="C20" s="2">
-        <v>300000</v>
+        <v>360000</v>
       </c>
       <c r="D20"/>
     </row>
@@ -320,7 +320,7 @@
         </is>
       </c>
       <c r="C21" s="2">
-        <v>300000</v>
+        <v>360000</v>
       </c>
       <c r="D21"/>
     </row>
@@ -332,7 +332,7 @@
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="4">
-        <v>7006600</v>
+        <v>6338000</v>
       </c>
       <c r="D22" s="1"/>
     </row>
@@ -367,7 +367,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-401</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="B35"/>
       <c r="C35" s="2">
-        <v>618000</v>
+        <v>617000</v>
       </c>
       <c r="D35"/>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="B50" s="1"/>
       <c r="C50" s="4">
-        <v>4511000</v>
+        <v>4510000</v>
       </c>
       <c r="D50" s="1"/>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B51" s="1"/>
       <c r="C51" s="4">
-        <v>31891000</v>
+        <v>31890000</v>
       </c>
       <c r="D51" s="1"/>
     </row>
@@ -681,7 +681,7 @@
       </c>
       <c r="B52" s="1"/>
       <c r="C52" s="4">
-        <v>5626600</v>
+        <v>4958000</v>
       </c>
       <c r="D52" s="1"/>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="B53" s="1"/>
       <c r="C53" s="4">
-        <v>1115600</v>
+        <v>448000</v>
       </c>
       <c r="D53" s="1"/>
     </row>
@@ -712,7 +712,7 @@
       </c>
       <c r="B55"/>
       <c r="C55" s="3">
-        <v>0.0338</v>
+        <v>0.0139</v>
       </c>
       <c r="D55"/>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B56"/>
       <c r="C56" s="3">
-        <v>0.1705</v>
+        <v>0.1533</v>
       </c>
       <c r="D56"/>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="B57"/>
       <c r="C57" s="3">
-        <v>0.0407</v>
+        <v>0.0164</v>
       </c>
       <c r="D57"/>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="B58"/>
       <c r="C58" s="3">
-        <v>0.1983</v>
+        <v>0.0904</v>
       </c>
       <c r="D58"/>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="B59"/>
       <c r="C59" s="2">
-        <v>5.6679</v>
+        <v>6.432</v>
       </c>
       <c r="D59"/>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="B60"/>
       <c r="C60" s="3">
-        <v>0.8295</v>
+        <v>0.8467</v>
       </c>
       <c r="D60"/>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="B61"/>
       <c r="C61" s="3">
-        <v>0.1367</v>
+        <v>0.1395</v>
       </c>
       <c r="D61"/>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="B62"/>
       <c r="C62" s="3">
-        <v>0.9662</v>
+        <v>0.9861</v>
       </c>
       <c r="D62"/>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="B63"/>
       <c r="C63" s="3">
-        <v>0.5766</v>
+        <v>0.5765</v>
       </c>
       <c r="D63"/>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="B66"/>
       <c r="C66" s="2">
-        <v>1.1338</v>
+        <v>1.0256</v>
       </c>
       <c r="D66"/>
     </row>
@@ -878,14 +878,14 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">BẢNG CHIA CỔ PHẦN CẦU GIẤY · kỳ 09/2026</t>
+          <t xml:space="preserve">BẢNG CHIA CỔ PHẦN T17 · kỳ 09/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Bản BC04-202609-CG-v1 · v1 · tạo 2026-10-06 09:00 bởi Hoàng Thu Hà · MAU-G1 · v1 (G1.31.8.26.xlsx) · RPT-ENGINE v1 · pnl.js schema 12 · Vốn = tỷ lệ × tiền thuê nhà kỳ; Tổng nhận = Vốn + LN ròng (R-08, D-07 chưa chốt)</t>
+          <t xml:space="preserve">Bản BC04-202609-T17-v1 · v1 · tạo 2026-10-06 09:00 bởi Hoàng Thu Hà · MAU-G1 · v1 (G1.31.8.26.xlsx) · RPT-ENGINE v1 · pnl.js schema 12 · Vốn = tỷ lệ × tiền thuê nhà kỳ; Tổng nhận = Vốn + LN ròng (R-08, D-07 chưa chốt)</t>
         </is>
       </c>
     </row>
@@ -935,13 +935,13 @@
         <v>7200000</v>
       </c>
       <c r="D5" s="2">
-        <v>2250640</v>
+        <v>1983200</v>
       </c>
       <c r="E5" s="2">
-        <v>446240</v>
+        <v>179200</v>
       </c>
       <c r="F5" s="2">
-        <v>7646240</v>
+        <v>7379200</v>
       </c>
     </row>
     <row r="6">
@@ -957,13 +957,13 @@
         <v>6300000</v>
       </c>
       <c r="D6" s="2">
-        <v>1969310</v>
+        <v>1735300</v>
       </c>
       <c r="E6" s="2">
-        <v>390460</v>
+        <v>156800</v>
       </c>
       <c r="F6" s="2">
-        <v>6690460</v>
+        <v>6456800</v>
       </c>
     </row>
     <row r="7">
@@ -979,13 +979,13 @@
         <v>4500000</v>
       </c>
       <c r="D7" s="2">
-        <v>1406650</v>
+        <v>1239500</v>
       </c>
       <c r="E7" s="2">
-        <v>278900</v>
+        <v>112000</v>
       </c>
       <c r="F7" s="2">
-        <v>4778900</v>
+        <v>4612000</v>
       </c>
     </row>
     <row r="8">
@@ -1001,13 +1001,13 @@
         <v>18000000</v>
       </c>
       <c r="D8" s="4">
-        <v>5626600</v>
+        <v>4958000</v>
       </c>
       <c r="E8" s="4">
-        <v>1115600</v>
+        <v>448000</v>
       </c>
       <c r="F8" s="4">
-        <v>19115600</v>
+        <v>18448000</v>
       </c>
     </row>
   </sheetData>
@@ -1029,14 +1029,14 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Nguồn từng dòng · TimeHouse Cầu Giấy · kỳ 09/2026</t>
+          <t xml:space="preserve">Nguồn từng dòng · Tòa T17 · Cầu Giấy · kỳ 09/2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Bản BC04-202609-CG-v1 · v1 · tạo 2026-10-06 09:00 bởi Hoàng Thu Hà · MAU-G1 · v1 (G1.31.8.26.xlsx) · RPT-ENGINE v1 · pnl.js schema 12 · nguồn tại thời điểm tạo báo cáo</t>
+          <t xml:space="preserve">Bản BC04-202609-T17-v1 · v1 · tạo 2026-10-06 09:00 bởi Hoàng Thu Hà · MAU-G1 · v1 (G1.31.8.26.xlsx) · RPT-ENGINE v1 · pnl.js schema 12 · nguồn tại thời điểm tạo báo cáo</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-401</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-401</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1166,12 +1166,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-401</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-401</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG101</t>
+          <t xml:space="preserve">INV-2609-101T17</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-101</t>
+          <t xml:space="preserve">101T17</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1234,12 +1234,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG102</t>
+          <t xml:space="preserve">INV-2609-102T17</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-102</t>
+          <t xml:space="preserve">102T17</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1269,12 +1269,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG201</t>
+          <t xml:space="preserve">INV-2609-201T17</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-201</t>
+          <t xml:space="preserve">201T17</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG202</t>
+          <t xml:space="preserve">INV-2609-202T17</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-202</t>
+          <t xml:space="preserve">202T17</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1339,12 +1339,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG301</t>
+          <t xml:space="preserve">INV-2609-301T17</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-301</t>
+          <t xml:space="preserve">301T17</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1374,12 +1374,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG302</t>
+          <t xml:space="preserve">INV-2609-302T17</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-302</t>
+          <t xml:space="preserve">302T17</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1409,21 +1409,21 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG101</t>
+          <t xml:space="preserve">INV-2609-101T17</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-101</t>
+          <t xml:space="preserve">101T17</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện (1678 → 1855) 672.600 ₫</t>
+          <t xml:space="preserve">Điện (1678 → 1855) 708.000 ₫</t>
         </is>
       </c>
       <c r="G14" s="2">
-        <v>672600</v>
+        <v>708000</v>
       </c>
     </row>
     <row r="15">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1444,21 +1444,21 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG102</t>
+          <t xml:space="preserve">INV-2609-102T17</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-102</t>
+          <t xml:space="preserve">102T17</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện (1904 → 2023) 452.200 ₫</t>
+          <t xml:space="preserve">Điện (1904 → 2023) 476.000 ₫</t>
         </is>
       </c>
       <c r="G15" s="2">
-        <v>452200</v>
+        <v>476000</v>
       </c>
     </row>
     <row r="16">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1479,21 +1479,21 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG201</t>
+          <t xml:space="preserve">INV-2609-201T17</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-201</t>
+          <t xml:space="preserve">201T17</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện (2035 → 2191) 592.800 ₫</t>
+          <t xml:space="preserve">Điện (2035 → 2191) 624.000 ₫</t>
         </is>
       </c>
       <c r="G16" s="2">
-        <v>592800</v>
+        <v>624000</v>
       </c>
     </row>
     <row r="17">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1514,21 +1514,21 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG202</t>
+          <t xml:space="preserve">INV-2609-202T17</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-202</t>
+          <t xml:space="preserve">202T17</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện (2261 → 2359) 372.400 ₫</t>
+          <t xml:space="preserve">Điện (2261 → 2359) 392.000 ₫</t>
         </is>
       </c>
       <c r="G17" s="2">
-        <v>372400</v>
+        <v>392000</v>
       </c>
     </row>
     <row r="18">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1549,21 +1549,21 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG301</t>
+          <t xml:space="preserve">INV-2609-301T17</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-301</t>
+          <t xml:space="preserve">301T17</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện (2392 → 2527) 513.000 ₫</t>
+          <t xml:space="preserve">Điện (2392 → 2527) 540.000 ₫</t>
         </is>
       </c>
       <c r="G18" s="2">
-        <v>513000</v>
+        <v>540000</v>
       </c>
     </row>
     <row r="19">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1584,21 +1584,21 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG302</t>
+          <t xml:space="preserve">INV-2609-302T17</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-302</t>
+          <t xml:space="preserve">302T17</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện (2618 → 2790) 653.600 ₫</t>
+          <t xml:space="preserve">Điện (2618 → 2790) 688.000 ₫</t>
         </is>
       </c>
       <c r="G19" s="2">
-        <v>653600</v>
+        <v>688000</v>
       </c>
     </row>
     <row r="20">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG101</t>
+          <t xml:space="preserve">INV-2609-101T17</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-101</t>
+          <t xml:space="preserve">101T17</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nước (322 → 326) 120.000 ₫</t>
+          <t xml:space="preserve">Nước (theo người) 120.000 ₫</t>
         </is>
       </c>
       <c r="G20" s="2">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1654,21 +1654,21 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG102</t>
+          <t xml:space="preserve">INV-2609-102T17</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-102</t>
+          <t xml:space="preserve">102T17</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nước (349 → 358) 270.000 ₫</t>
+          <t xml:space="preserve">Nước (theo người) 240.000 ₫</t>
         </is>
       </c>
       <c r="G21" s="2">
-        <v>270000</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="22">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1689,21 +1689,21 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG201</t>
+          <t xml:space="preserve">INV-2609-201T17</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-201</t>
+          <t xml:space="preserve">201T17</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nước (364 → 372) 240.000 ₫</t>
+          <t xml:space="preserve">Nước (theo người) 120.000 ₫</t>
         </is>
       </c>
       <c r="G22" s="2">
-        <v>240000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="23">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1724,21 +1724,21 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG202</t>
+          <t xml:space="preserve">INV-2609-202T17</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-202</t>
+          <t xml:space="preserve">202T17</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nước (379 → 386) 210.000 ₫</t>
+          <t xml:space="preserve">Nước (theo người) 240.000 ₫</t>
         </is>
       </c>
       <c r="G23" s="2">
-        <v>210000</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="24">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1759,21 +1759,21 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG301</t>
+          <t xml:space="preserve">INV-2609-301T17</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-301</t>
+          <t xml:space="preserve">301T17</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nước (406 → 412) 180.000 ₫</t>
+          <t xml:space="preserve">Nước (theo người) 120.000 ₫</t>
         </is>
       </c>
       <c r="G24" s="2">
-        <v>180000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="25">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1794,21 +1794,21 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG302</t>
+          <t xml:space="preserve">INV-2609-302T17</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-302</t>
+          <t xml:space="preserve">302T17</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nước (421 → 426) 150.000 ₫</t>
+          <t xml:space="preserve">Nước (theo người) 240.000 ₫</t>
         </is>
       </c>
       <c r="G25" s="2">
-        <v>150000</v>
+        <v>240000</v>
       </c>
     </row>
     <row r="26">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1829,21 +1829,21 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG101</t>
+          <t xml:space="preserve">INV-2609-101T17</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-101</t>
+          <t xml:space="preserve">101T17</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G26" s="2">
-        <v>50000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="27">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1864,21 +1864,21 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG102</t>
+          <t xml:space="preserve">INV-2609-102T17</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-102</t>
+          <t xml:space="preserve">102T17</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G27" s="2">
-        <v>50000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="28">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1899,21 +1899,21 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG201</t>
+          <t xml:space="preserve">INV-2609-201T17</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-201</t>
+          <t xml:space="preserve">201T17</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G28" s="2">
-        <v>50000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="29">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1934,21 +1934,21 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG202</t>
+          <t xml:space="preserve">INV-2609-202T17</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-202</t>
+          <t xml:space="preserve">202T17</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G29" s="2">
-        <v>50000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="30">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1969,21 +1969,21 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG301</t>
+          <t xml:space="preserve">INV-2609-301T17</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-301</t>
+          <t xml:space="preserve">301T17</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G30" s="2">
-        <v>50000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="31">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2004,21 +2004,21 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG302</t>
+          <t xml:space="preserve">INV-2609-302T17</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-302</t>
+          <t xml:space="preserve">302T17</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G31" s="2">
-        <v>50000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="32">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2039,12 +2039,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG101</t>
+          <t xml:space="preserve">INV-2609-101T17</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-101</t>
+          <t xml:space="preserve">101T17</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2074,12 +2074,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG102</t>
+          <t xml:space="preserve">INV-2609-102T17</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-102</t>
+          <t xml:space="preserve">102T17</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2109,12 +2109,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG201</t>
+          <t xml:space="preserve">INV-2609-201T17</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-201</t>
+          <t xml:space="preserve">201T17</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG202</t>
+          <t xml:space="preserve">INV-2609-202T17</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-202</t>
+          <t xml:space="preserve">202T17</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2179,12 +2179,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG301</t>
+          <t xml:space="preserve">INV-2609-301T17</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-301</t>
+          <t xml:space="preserve">301T17</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2214,12 +2214,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG302</t>
+          <t xml:space="preserve">INV-2609-302T17</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-302</t>
+          <t xml:space="preserve">302T17</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2249,32 +2249,32 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG101</t>
+          <t xml:space="preserve">INV-2609-301T17</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-101</t>
+          <t xml:space="preserve">301T17</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gửi xe điện 120.000 ₫</t>
+          <t xml:space="preserve">Gửi xe đạp điện 150.000 ₫</t>
         </is>
       </c>
       <c r="G38" s="2">
-        <v>120000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu xe điện</t>
+          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2284,32 +2284,32 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG102</t>
+          <t xml:space="preserve">INV-2609-101T17</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-102</t>
+          <t xml:space="preserve">101T17</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gửi xe điện 240.000 ₫</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G39" s="2">
-        <v>240000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu xe điện</t>
+          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2319,32 +2319,32 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG201</t>
+          <t xml:space="preserve">INV-2609-102T17</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-201</t>
+          <t xml:space="preserve">102T17</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gửi xe điện 120.000 ₫</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G40" s="2">
-        <v>120000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu xe điện</t>
+          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2354,32 +2354,32 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG202</t>
+          <t xml:space="preserve">INV-2609-201T17</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-202</t>
+          <t xml:space="preserve">201T17</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gửi xe điện 240.000 ₫</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G41" s="2">
-        <v>240000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu xe điện</t>
+          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2389,32 +2389,32 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG301</t>
+          <t xml:space="preserve">INV-2609-202T17</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-301</t>
+          <t xml:space="preserve">202T17</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gửi xe điện 120.000 ₫</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G42" s="2">
-        <v>120000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu xe điện</t>
+          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2424,21 +2424,21 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG302</t>
+          <t xml:space="preserve">INV-2609-301T17</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-302</t>
+          <t xml:space="preserve">301T17</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gửi xe điện 240.000 ₫</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G43" s="2">
-        <v>240000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="44">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2459,32 +2459,32 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG101</t>
+          <t xml:space="preserve">INV-2609-302T17</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-101</t>
+          <t xml:space="preserve">302T17</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G44" s="2">
-        <v>50000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
+          <t xml:space="preserve">Doanh thu máy giặt</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2494,32 +2494,32 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG102</t>
+          <t xml:space="preserve">INV-2609-101T17</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-102</t>
+          <t xml:space="preserve">101T17</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G45" s="2">
-        <v>50000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
+          <t xml:space="preserve">Doanh thu máy giặt</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2529,32 +2529,32 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG201</t>
+          <t xml:space="preserve">INV-2609-102T17</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-201</t>
+          <t xml:space="preserve">102T17</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G46" s="2">
-        <v>50000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
+          <t xml:space="preserve">Doanh thu máy giặt</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2564,32 +2564,32 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG202</t>
+          <t xml:space="preserve">INV-2609-201T17</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-202</t>
+          <t xml:space="preserve">201T17</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G47" s="2">
-        <v>50000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
+          <t xml:space="preserve">Doanh thu máy giặt</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2599,32 +2599,32 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG301</t>
+          <t xml:space="preserve">INV-2609-202T17</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-301</t>
+          <t xml:space="preserve">202T17</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G48" s="2">
-        <v>50000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu phí thang máy / DV khác</t>
+          <t xml:space="preserve">Doanh thu máy giặt</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2634,21 +2634,21 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG302</t>
+          <t xml:space="preserve">INV-2609-301T17</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-302</t>
+          <t xml:space="preserve">301T17</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 40.000 ₫ (1/3 phí DV chung 120.000 ₫)</t>
         </is>
       </c>
       <c r="G49" s="2">
-        <v>50000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="50">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2669,207 +2669,191 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG101</t>
+          <t xml:space="preserve">INV-2609-302T17</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-101</t>
+          <t xml:space="preserve">302T17</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Dịch vụ chung 80.000 ₫ (1/3 phí DV chung 240.000 ₫)</t>
         </is>
       </c>
       <c r="G50" s="2">
-        <v>50000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu máy giặt</t>
+          <t xml:space="preserve">Tiền thuê nhà 1 tháng</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hóa đơn</t>
+          <t xml:space="preserve">Chi phí</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG102</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CG-102</t>
-        </is>
-      </c>
+          <t xml:space="preserve">CP-2609-067</t>
+        </is>
+      </c>
+      <c r="E51"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Tiền thuê trả chủ nhà · Tiền thuê tòa tháng 09/2026 · HĐTT-T17-09</t>
         </is>
       </c>
       <c r="G51" s="2">
-        <v>50000</v>
+        <v>18000000</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu máy giặt</t>
+          <t xml:space="preserve">Mua sắm thêm thiết bị</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hóa đơn</t>
+          <t xml:space="preserve">Chi phí</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG201</t>
+          <t xml:space="preserve">CP-2609-108</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">CG-201</t>
+          <t xml:space="preserve">401T17</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Mua sắm thiết bị · Tủ lạnh + rèm phòng 401T17 · HĐ10963</t>
         </is>
       </c>
       <c r="G52" s="2">
-        <v>50000</v>
+        <v>3200000</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu máy giặt</t>
+          <t xml:space="preserve">Điện</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hóa đơn</t>
+          <t xml:space="preserve">Chi phí</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG202</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CG-202</t>
-        </is>
-      </c>
+          <t xml:space="preserve">CP-2609-068</t>
+        </is>
+      </c>
+      <c r="E53"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Điện nước tổng (công tơ nguồn) · Hóa đơn điện nước công tơ tổng · HĐ10683</t>
         </is>
       </c>
       <c r="G53" s="2">
-        <v>50000</v>
+        <v>3264000</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu máy giặt</t>
+          <t xml:space="preserve">Nước</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hóa đơn</t>
+          <t xml:space="preserve">Chi phí</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG301</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CG-301</t>
-        </is>
-      </c>
+          <t xml:space="preserve">CP-2609-068</t>
+        </is>
+      </c>
+      <c r="E54"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Điện nước tổng (công tơ nguồn) · Hóa đơn điện nước công tơ tổng · HĐ10683</t>
         </is>
       </c>
       <c r="G54" s="2">
-        <v>50000</v>
+        <v>816000</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu máy giặt</t>
+          <t xml:space="preserve">Mạng</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hóa đơn</t>
+          <t xml:space="preserve">Chi phí</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">INV-2609-CG302</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CG-302</t>
-        </is>
-      </c>
+          <t xml:space="preserve">CP-2609-070</t>
+        </is>
+      </c>
+      <c r="E55"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí dịch vụ 50.000 ₫ (1/3 phí DV chung 150.000 ₫)</t>
+          <t xml:space="preserve">Internet / truyền hình · Internet cáp quang toàn tòa · HĐ10697</t>
         </is>
       </c>
       <c r="G55" s="2">
-        <v>50000</v>
+        <v>1100000</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiền thuê nhà 1 tháng</t>
+          <t xml:space="preserve">Phí thu rác</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2879,28 +2863,28 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP-2609-067</t>
+          <t xml:space="preserve">CP-2609-069</t>
         </is>
       </c>
       <c r="E56"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiền thuê trả chủ nhà · Tiền thuê tòa tháng 09/2026 · HĐTT-CG-09</t>
+          <t xml:space="preserve">Phí thu rác / môi trường · Phí thu gom rác tháng 09 · HĐ10690</t>
         </is>
       </c>
       <c r="G56" s="2">
-        <v>18000000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mua sắm thêm thiết bị</t>
+          <t xml:space="preserve">Phí bảo trì thang máy</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2910,249 +2894,245 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP-2609-108</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CG-401</t>
-        </is>
-      </c>
+          <t xml:space="preserve">CP-2609-104</t>
+        </is>
+      </c>
+      <c r="E57"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mua sắm thiết bị · Tủ lạnh + rèm phòng CG-401 · HĐ10963</t>
+          <t xml:space="preserve">Bảo trì thang máy · Bảo trì thang máy định kỳ quý 3 · HĐ10935</t>
         </is>
       </c>
       <c r="G57" s="2">
-        <v>3200000</v>
+        <v>800000</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện</t>
+          <t xml:space="preserve">Lương quản lý</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chi phí</t>
+          <t xml:space="preserve">Lương</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP-2609-068</t>
+          <t xml:space="preserve">NV-003</t>
         </is>
       </c>
       <c r="E58"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện nước tổng (công tơ nguồn) · Hóa đơn điện nước công tơ tổng · HĐ10683</t>
+          <t xml:space="preserve">Vũ Quang Huy · HS 72,1% × 7 phòng</t>
         </is>
       </c>
       <c r="G58" s="2">
-        <v>3264000</v>
+        <v>617000</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nước</t>
+          <t xml:space="preserve">Lương quản lý tổng</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chi phí</t>
+          <t xml:space="preserve">Phân bổ chung</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP-2609-068</t>
+          <t xml:space="preserve">gm</t>
         </is>
       </c>
       <c r="E59"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Điện nước tổng (công tơ nguồn) · Hóa đơn điện nước công tơ tổng · HĐ10683</t>
+          <t xml:space="preserve">252.000 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G59" s="2">
-        <v>816000</v>
+        <v>98000</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mạng</t>
+          <t xml:space="preserve">Lương trưởng phòng vận hành</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chi phí</t>
+          <t xml:space="preserve">Phân bổ chung</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP-2609-070</t>
+          <t xml:space="preserve">opsHead</t>
         </is>
       </c>
       <c r="E60"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internet / truyền hình · Internet cáp quang toàn tòa · HĐ10697</t>
+          <t xml:space="preserve">270.000 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G60" s="2">
-        <v>1100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí thu rác</t>
+          <t xml:space="preserve">Lương trưởng nhóm vận hành</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chi phí</t>
+          <t xml:space="preserve">Lương</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP-2609-069</t>
+          <t xml:space="preserve">NV-003</t>
         </is>
       </c>
       <c r="E61"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí thu rác / môi trường · Phí thu gom rác tháng 09 · HĐ10690</t>
+          <t xml:space="preserve">Vũ Quang Huy · 7 phòng × 10.000 ₫</t>
         </is>
       </c>
       <c r="G61" s="2">
-        <v>200000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí bảo trì thang máy</t>
+          <t xml:space="preserve">Lương nhân viên nguồn</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chi phí</t>
+          <t xml:space="preserve">Phân bổ chung</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP-2609-104</t>
+          <t xml:space="preserve">source</t>
         </is>
       </c>
       <c r="E62"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bảo trì thang máy · Bảo trì thang máy định kỳ quý 3 · HĐ10935</t>
+          <t xml:space="preserve">90.000 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G62" s="2">
-        <v>800000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương quản lý</t>
+          <t xml:space="preserve">Lương NVKD</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương</t>
+          <t xml:space="preserve">Phân bổ chung</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">NV-003</t>
+          <t xml:space="preserve">sales</t>
         </is>
       </c>
       <c r="E63"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vũ Quang Huy · HS 72,3% × 7 phòng</t>
+          <t xml:space="preserve">180.000 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G63" s="2">
-        <v>618000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương quản lý tổng</t>
+          <t xml:space="preserve">Lương vệ sinh</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phân bổ chung</t>
+          <t xml:space="preserve">Chi phí</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">gm</t>
+          <t xml:space="preserve">CP-2609-071</t>
         </is>
       </c>
       <c r="E64"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t xml:space="preserve">252.000 ₫ × 7/18 phòng</t>
+          <t xml:space="preserve">Vệ sinh · Vệ sinh khu chung · HĐ10704</t>
         </is>
       </c>
       <c r="G64" s="2">
-        <v>98000</v>
+        <v>1500000</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương trưởng phòng vận hành</t>
+          <t xml:space="preserve">Lương kế toán</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3162,59 +3142,59 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">opsHead</t>
+          <t xml:space="preserve">acct</t>
         </is>
       </c>
       <c r="E65"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">270.000 ₫ × 7/18 phòng</t>
+          <t xml:space="preserve">180.000 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G65" s="2">
-        <v>105000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương trưởng nhóm vận hành</t>
+          <t xml:space="preserve">Lương sửa chữa</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương</t>
+          <t xml:space="preserve">Phân bổ chung</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">NV-003</t>
+          <t xml:space="preserve">repairStaff</t>
         </is>
       </c>
       <c r="E66"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vũ Quang Huy · 7 phòng × 10.000 ₫</t>
+          <t xml:space="preserve">90.000 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G66" s="2">
-        <v>70000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương nhân viên nguồn</t>
+          <t xml:space="preserve">Lương bảo vệ</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3224,28 +3204,28 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">source</t>
+          <t xml:space="preserve">security</t>
         </is>
       </c>
       <c r="E67"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">90.000 ₫ × 7/18 phòng</t>
+          <t xml:space="preserve">0 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G67" s="2">
-        <v>35000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương NVKD</t>
+          <t xml:space="preserve">Thuê và DV văn phòng</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3255,233 +3235,78 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">sales</t>
+          <t xml:space="preserve">office</t>
         </is>
       </c>
       <c r="E68"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">180.000 ₫ × 7/18 phòng</t>
+          <t xml:space="preserve">360.000 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G68" s="2">
-        <v>70000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương vệ sinh</t>
+          <t xml:space="preserve">Phí marketing / hoa hồng</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chi phí</t>
+          <t xml:space="preserve">Phân bổ chung</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">CP-2609-071</t>
+          <t xml:space="preserve">marketing</t>
         </is>
       </c>
       <c r="E69"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vệ sinh · Vệ sinh khu chung · HĐ10704</t>
+          <t xml:space="preserve">180.000 ₫ × 7/18 phòng</t>
         </is>
       </c>
       <c r="G69" s="2">
-        <v>1500000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lương kế toán</t>
+          <t xml:space="preserve">Sửa chữa, thay thế, bảo trì</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Giấy</t>
+          <t xml:space="preserve">T17</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phân bổ chung</t>
+          <t xml:space="preserve">Chi phí</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">acct</t>
+          <t xml:space="preserve">CP-2609-072</t>
         </is>
       </c>
       <c r="E70"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t xml:space="preserve">180.000 ₫ × 7/18 phòng</t>
+          <t xml:space="preserve">Sửa chữa, bảo trì · Sửa khóa cửa · HĐ10711</t>
         </is>
       </c>
       <c r="G70" s="2">
-        <v>70000</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lương sửa chữa</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cầu Giấy</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phân bổ chung</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">repairStaff</t>
-        </is>
-      </c>
-      <c r="E71"/>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">90.000 ₫ × 7/18 phòng</t>
-        </is>
-      </c>
-      <c r="G71" s="2">
-        <v>35000</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lương bảo vệ</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cầu Giấy</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phân bổ chung</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">security</t>
-        </is>
-      </c>
-      <c r="E72"/>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0 ₫ × 7/18 phòng</t>
-        </is>
-      </c>
-      <c r="G72" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Thuê và DV văn phòng</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cầu Giấy</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phân bổ chung</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">office</t>
-        </is>
-      </c>
-      <c r="E73"/>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">360.000 ₫ × 7/18 phòng</t>
-        </is>
-      </c>
-      <c r="G73" s="2">
-        <v>140000</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phí marketing / hoa hồng</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cầu Giấy</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Phân bổ chung</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">marketing</t>
-        </is>
-      </c>
-      <c r="E74"/>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">180.000 ₫ × 7/18 phòng</t>
-        </is>
-      </c>
-      <c r="G74" s="2">
-        <v>70000</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sửa chữa, thay thế, bảo trì</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cầu Giấy</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chi phí</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CP-2609-072</t>
-        </is>
-      </c>
-      <c r="E75"/>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sửa chữa, bảo trì · Sửa khóa cửa · HĐ10711</t>
-        </is>
-      </c>
-      <c r="G75" s="2">
         <v>1700000</v>
       </c>
     </row>
@@ -3507,7 +3332,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="6">
         <is>
-          <t xml:space="preserve">Bản BC04-202609-CG-v1 · v1 · tạo 2026-10-06 09:00 bởi Hoàng Thu Hà · MAU-G1 · v1 (G1.31.8.26.xlsx) · RPT-ENGINE v1 · pnl.js schema 12</t>
+          <t xml:space="preserve">Bản BC04-202609-T17-v1 · v1 · tạo 2026-10-06 09:00 bởi Hoàng Thu Hà · MAU-G1 · v1 (G1.31.8.26.xlsx) · RPT-ENGINE v1 · pnl.js schema 12</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3688,11 @@
           <t xml:space="preserve">DT tiền phòng + DT dịch vụ + cọc phòng mới + cọc khách bỏ − hoàn cọc</t>
         </is>
       </c>
-      <c r="C24"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3876,7 +3705,11 @@
           <t xml:space="preserve">Điện + nước + vệ sinh + mạng + xe điện + thang máy/DV khác + máy giặt</t>
         </is>
       </c>
-      <c r="C25"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3889,7 +3722,11 @@
           <t xml:space="preserve">Giá gốc dịch vụ: điện + nước + mạng + thu rác + môi trường + thang máy</t>
         </is>
       </c>
-      <c r="C26"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3902,7 +3739,11 @@
           <t xml:space="preserve">Tiền thuê nhà + mua sắm thiết bị + giá gốc dịch vụ</t>
         </is>
       </c>
-      <c r="C27"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3915,7 +3756,11 @@
           <t xml:space="preserve">Tổng các dòng lương</t>
         </is>
       </c>
-      <c r="C28"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3928,7 +3773,11 @@
           <t xml:space="preserve">Lương + thuê/DV văn phòng + marketing/hoa hồng + sửa chữa + chi phí khác</t>
         </is>
       </c>
-      <c r="C29"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3941,7 +3790,11 @@
           <t xml:space="preserve">Giá vốn + chi phí bán hàng</t>
         </is>
       </c>
-      <c r="C30"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3954,7 +3807,11 @@
           <t xml:space="preserve">Doanh thu − giá vốn</t>
         </is>
       </c>
-      <c r="C31"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3967,7 +3824,11 @@
           <t xml:space="preserve">Doanh thu − tổng chi phí</t>
         </is>
       </c>
-      <c r="C32"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chuẩn</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3977,7 +3838,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lợi nhuận ròng (LNR) ÷ Tổng doanh thu tháng</t>
+          <t xml:space="preserve">(Lợi nhuận ròng (LNR)) ÷ (Tổng doanh thu tháng)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3994,7 +3855,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lợi nhuận gộp (LNG) ÷ Tổng doanh thu tháng</t>
+          <t xml:space="preserve">(Lợi nhuận gộp (LNG)) ÷ (Tổng doanh thu tháng)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4011,7 +3872,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lợi nhuận ròng (LNR) ÷ Giá vốn (GV)</t>
+          <t xml:space="preserve">(Lợi nhuận ròng (LNR)) ÷ (Giá vốn (GV))</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4028,7 +3889,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lợi nhuận ròng (LNR) ÷ Lợi nhuận gộp (LNG)</t>
+          <t xml:space="preserve">(Lợi nhuận ròng (LNR)) ÷ (Lợi nhuận gộp (LNG))</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4045,7 +3906,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">TỔNG CHI PHÍ (TCP) ÷ Lợi nhuận gộp (LNG)</t>
+          <t xml:space="preserve">(TỔNG CHI PHÍ (TCP)) ÷ (Lợi nhuận gộp (LNG))</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4062,7 +3923,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Giá vốn (GV) ÷ Tổng doanh thu tháng</t>
+          <t xml:space="preserve">(Giá vốn (GV)) ÷ (Tổng doanh thu tháng)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4079,7 +3940,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tổng chi phí bán hàng (CPBH) ÷ Tổng doanh thu tháng</t>
+          <t xml:space="preserve">(Tổng chi phí bán hàng (CPBH)) ÷ (Tổng doanh thu tháng)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4096,7 +3957,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">TỔNG CHI PHÍ (TCP) ÷ Tổng doanh thu tháng</t>
+          <t xml:space="preserve">(TỔNG CHI PHÍ (TCP)) ÷ (Tổng doanh thu tháng)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4113,7 +3974,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tổng lương ÷ Tổng chi phí bán hàng (CPBH)</t>
+          <t xml:space="preserve">(Tổng lương) ÷ (Tổng chi phí bán hàng (CPBH))</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4130,7 +3991,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phí marketing / hoa hồng ÷ Tổng chi phí bán hàng (CPBH)</t>
+          <t xml:space="preserve">(Phí marketing / hoa hồng) ÷ (Tổng chi phí bán hàng (CPBH))</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4147,7 +4008,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chi phí khác ÷ Tổng chi phí bán hàng (CPBH)</t>
+          <t xml:space="preserve">(Chi phí khác) ÷ (Tổng chi phí bán hàng (CPBH))</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4164,7 +4025,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu tổng dịch vụ nhà ÷ Giá gốc dịch vụ (tổng)</t>
+          <t xml:space="preserve">(Doanh thu tổng dịch vụ nhà) ÷ (Giá gốc dịch vụ (tổng))</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -4181,7 +4042,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Doanh thu tiền phòng ÷ Tiền thuê nhà 1 tháng</t>
+          <t xml:space="preserve">(Doanh thu tiền phòng) ÷ (Tiền thuê nhà 1 tháng)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">

</xml_diff>